<commit_message>
feat(evaluation): preparar estudios por pares y jueces de preferencias
- Añadir estudios SQLite, congelación, asignaciones y votos persistentes.
- Integrar /evaluar, /aportar y /pausa en Telegram.
- Incorporar extracción de rasgos con evidencias, caché e informes.
- Añadir Bradley-Terry y tres jueces con validación fuera de muestra.
- Preparar baseline directo, rankings y fichas de análisis.
- Actualizar metodología, catálogo, planilla y guía operativa.
- Documentar los pendientes detectados en la auditoría del tutor.

Validación previa: quality.ps1 limpio; 755 pruebas pasadas y 2 omitidas.
Demo: 11 historias ficticias, 180 respuestas y ninguna llamada de red.
Actualización documental: git diff --check limpio.

Quedan pendientes la integración de extracciones del estudio con informes,
ajustes de recuento y compatibilidad, y la validación experimental real.
No se genera el corpus definitivo ni se modifica la simulación.
</commit_message>
<xml_diff>
--- a/packages/evaluation/planilla/planilla_evaluacion.xlsx
+++ b/packages/evaluation/planilla/planilla_evaluacion.xlsx
@@ -433,7 +433,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -813,7 +813,7 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
@@ -895,7 +895,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -977,7 +977,7 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1054,7 +1054,7 @@
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1136,7 +1136,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1218,7 +1218,7 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1295,7 +1295,7 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1459,7 +1459,7 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1536,7 +1536,7 @@
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1613,7 +1613,7 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -1695,7 +1695,7 @@
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -1767,7 +1767,7 @@
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -1844,7 +1844,7 @@
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -1916,7 +1916,7 @@
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -1988,7 +1988,7 @@
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
@@ -2060,7 +2060,7 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -2137,7 +2137,7 @@
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
@@ -2296,7 +2296,7 @@
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
@@ -2373,7 +2373,7 @@
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
@@ -2455,7 +2455,7 @@
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
@@ -2527,7 +2527,7 @@
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
@@ -2604,7 +2604,7 @@
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
@@ -2676,7 +2676,7 @@
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
@@ -2753,7 +2753,7 @@
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
@@ -2825,7 +2825,7 @@
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
@@ -2912,7 +2912,7 @@
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
@@ -2989,7 +2989,7 @@
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
@@ -3071,7 +3071,7 @@
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
@@ -3153,7 +3153,7 @@
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
@@ -3235,7 +3235,7 @@
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr">
@@ -3317,7 +3317,7 @@
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
@@ -3394,7 +3394,7 @@
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K41" s="2" t="inlineStr">
@@ -3481,7 +3481,7 @@
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr">
@@ -3558,7 +3558,7 @@
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr">
@@ -3630,7 +3630,7 @@
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
@@ -3712,7 +3712,7 @@
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K45" s="2" t="inlineStr">
@@ -3794,7 +3794,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -3876,7 +3876,7 @@
       </c>
       <c r="J47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K47" s="2" t="inlineStr">
@@ -3953,7 +3953,7 @@
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K48" s="2" t="inlineStr">
@@ -4025,7 +4025,7 @@
       </c>
       <c r="J49" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K49" s="2" t="inlineStr">
@@ -4107,7 +4107,7 @@
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K50" s="2" t="inlineStr">
@@ -4184,7 +4184,7 @@
       </c>
       <c r="J51" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K51" s="2" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K52" s="2" t="inlineStr">
@@ -4343,7 +4343,7 @@
       </c>
       <c r="J53" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K53" s="2" t="inlineStr">
@@ -4425,7 +4425,7 @@
       </c>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K54" s="2" t="inlineStr">
@@ -4507,7 +4507,7 @@
       </c>
       <c r="J55" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K55" s="2" t="inlineStr">
@@ -4589,7 +4589,7 @@
       </c>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K56" s="2" t="inlineStr">
@@ -4671,7 +4671,7 @@
       </c>
       <c r="J57" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K57" s="2" t="inlineStr">
@@ -4748,7 +4748,7 @@
       </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K58" s="2" t="inlineStr">
@@ -4825,7 +4825,7 @@
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr">
@@ -4907,7 +4907,7 @@
       </c>
       <c r="J60" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K60" s="2" t="inlineStr">
@@ -4989,7 +4989,7 @@
       </c>
       <c r="J61" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K61" s="2" t="inlineStr">
@@ -5066,7 +5066,7 @@
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K62" s="2" t="inlineStr">
@@ -5148,7 +5148,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr">
@@ -5235,7 +5235,7 @@
       </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K64" s="2" t="inlineStr">
@@ -9828,7 +9828,7 @@
       </c>
       <c r="J133" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K133" s="2" t="inlineStr">
@@ -9900,7 +9900,7 @@
       </c>
       <c r="J134" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K134" s="2" t="inlineStr">
@@ -9972,7 +9972,7 @@
       </c>
       <c r="J135" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K135" s="2" t="inlineStr">
@@ -10044,7 +10044,7 @@
       </c>
       <c r="J136" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K136" s="2" t="inlineStr">
@@ -10111,7 +10111,7 @@
       </c>
       <c r="J137" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K137" s="2" t="inlineStr">
@@ -10183,7 +10183,7 @@
       </c>
       <c r="J138" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K138" s="2" t="inlineStr">
@@ -10255,7 +10255,7 @@
       </c>
       <c r="J139" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K139" s="2" t="inlineStr">
@@ -10327,7 +10327,7 @@
       </c>
       <c r="J140" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">por_construir</t>
+          <t xml:space="preserve">existe</t>
         </is>
       </c>
       <c r="K140" s="2" t="inlineStr">

</xml_diff>